<commit_message>
craetion of standart table
</commit_message>
<xml_diff>
--- a/Projeto FINOS/microcontrolador_precos.xlsx
+++ b/Projeto FINOS/microcontrolador_precos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diogo\Documents\Projeto FINOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F6ECA3-DF54-42A8-BAB1-83DA86CAEAF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FD8709-4AF4-4417-956E-B22DAAABB008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="156" windowWidth="23040" windowHeight="12204" xr2:uid="{70A57D92-16A9-410E-AE88-7C626E365A8B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="73">
   <si>
     <t>board</t>
   </si>
@@ -59,9 +59,6 @@
     <t>https://pt.aliexpress.com/item/1005007671225942.html?spm=a2g0o.productlist.main.4.33bewbpBwbpB4d&amp;algo_pvid=8a0946c9-6135-4953-9734-6fb441ff5631&amp;algo_exp_id=8a0946c9-6135-4953-9734-6fb441ff5631-3&amp;pdp_ext_f=%7B%22order%22%3A%221743%22%2C%22eval%22%3A%221%22%7D&amp;pdp_npi=4%40dis%21EUR%214.83%214.38%21%21%2138.67%2135.07%21%402103867617488812947106565ec0ba%2112000042934077713%21sea%21PT%210%21ABX&amp;curPageLogUid=H76qrjBNJxjg&amp;utparam-url=scene%3Asearch%7Cquery_from%3A</t>
   </si>
   <si>
-    <t>https://pt.aliexpress.com/item/1005005097003947.html?spm=a2g0o.productlist.main.1.1f62Z1hhZ1hhOF&amp;algo_pvid=7620f411-5908-4f28-a721-fde32d87f1f0&amp;algo_exp_id=7620f411-5908-4f28-a721-fde32d87f1f0-0&amp;pdp_ext_f=%7B%22order%22%3A%222%22%2C%22eval%22%3A%221%22%7D&amp;pdp_npi=4%40dis%21EUR%2129.68%2128.19%21%21%2132.96%2131.31%21%40211b813f17488999111086659e9725%2112000032129741975%21sea%21PT%210%21ABX&amp;curPageLogUid=5Nm12r7Ngdme&amp;utparam-url=scene%3Asearch%7Cquery_from%3A</t>
-  </si>
-  <si>
     <t>leds and resistences</t>
   </si>
   <si>
@@ -110,12 +107,6 @@
     <t>BREADBOARD</t>
   </si>
   <si>
-    <t>load cell 5kg hx711</t>
-  </si>
-  <si>
-    <t>28,19hh</t>
-  </si>
-  <si>
     <t>n1,96</t>
   </si>
   <si>
@@ -206,13 +197,64 @@
     <t>https://pt.aliexpress.com/item/1005006361814667.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%204.13%21EUR%203.88%21%21EUR%203.88%21%21%21%402103919917516586444672403e92e2%2112000036895232315%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
   </si>
   <si>
-    <t>https://pt.aliexpress.com/item/1005006918669019.html?spm=a2g0o.detail.0.0.5d783Gua3Guaba&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%205.80%21EUR%200.88%21%21EUR%200.88%21%21%21%402103894417539156120946203e3b3f%2112000038723932736%21ct%21PT%21-1%21%211%210&amp;gatewayAdapt=glo2bra</t>
-  </si>
-  <si>
-    <t>https://pt.aliexpress.com/item/4000208456751.html?spm=a2g0o.detail.0.0.5d783Gua3Guaba&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.08%21EUR%200.88%21%21EUR%200.88%21%21%21%402103894417539156120946203e3b3f%2110000000799552169%21ct%21PT%21-1%21%211%210&amp;pdp_ext_f=%7B%22cart2PdpParams%22%3A%7B%22pdpBusinessMode%22%3A%22retail%22%7D%7D&amp;gatewayAdapt=glo2bra</t>
-  </si>
-  <si>
-    <t>https://pt.aliexpress.com/item/1005006897944758.html?spm=a2g0o.cart.0.0.379d7f06nRUJpj&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.07%21EUR%202.07%21%21EUR%202.07%21%21%21%402103894417539157290177387e3b3f%2112000038652696056%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
+    <t>https://pt.aliexpress.com/item/2036819167.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%2018.48%21EUR%2012.20%21%21EUR%2012.20%21%21%21%40211b61a417550327284106006edd2d%2167389781053%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1m 100 led /m </t>
+  </si>
+  <si>
+    <t>w2812b</t>
+  </si>
+  <si>
+    <t>https://pt.aliexpress.com/item/1005007205148171.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%205.07%21EUR%204.56%21%21EUR%204.56%21%21%21%40211b80f717550322996453403e26a5%2112000039796887787%21ct%21PT%216241319494%21%214%210&amp;gatewayAdapt=glo2bra</t>
+  </si>
+  <si>
+    <t>load cell hx711</t>
+  </si>
+  <si>
+    <t>https://pt.aliexpress.com/item/1005006897944758.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.07%21EUR%202.07%21%21EUR%202.07%21%21%21%40211b80f717550322996453403e26a5%2112000038652696056%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
+  </si>
+  <si>
+    <t>sot23-3 to sip3</t>
+  </si>
+  <si>
+    <t>https://pt.aliexpress.com/item/1005006142488372.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%204.26%21EUR%201.36%21%21EUR%201.36%21%21%21%40211b80f717550322996453403e26a5%2112000035951341855%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
+  </si>
+  <si>
+    <t>AO3401</t>
+  </si>
+  <si>
+    <t>https://pt.aliexpress.com/item/32866531235.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%203.05%21EUR%202.72%21%21EUR%202.72%21%21%21%40211b80f717550322996453403e26a5%2112000028848788987%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
+  </si>
+  <si>
+    <t>1N5822</t>
+  </si>
+  <si>
+    <t>https://pt.aliexpress.com/item/1005002524973878.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%201.85%21EUR%201.85%21%21EUR%201.85%21%21%21%40211b80f717550322996453403e26a5%2112000020995893453%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
+  </si>
+  <si>
+    <t>1000UF capacitor</t>
+  </si>
+  <si>
+    <t>https://pt.aliexpress.com/item/1005003252824475.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%204.37%21EUR%204.09%21%21EUR%204.09%21%21%21%40211b80f717550322996453403e26a5%2112000024867532534%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
+  </si>
+  <si>
+    <t>https://pt.aliexpress.com/item/1005004336218242.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%203.02%21EUR%203.02%21%21EUR%203.02%21%21%21%40211b80f717550322996453403e26a5%2112000028806929674%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
+  </si>
+  <si>
+    <t>10m</t>
+  </si>
+  <si>
+    <t>jumper cable 24awg</t>
+  </si>
+  <si>
+    <t>cabo 24 awg preto</t>
+  </si>
+  <si>
+    <t>cabo 24 awg red</t>
+  </si>
+  <si>
+    <t>https://pt.aliexpress.com/item/1005004336218242.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.99%21EUR%202.99%21%21EUR%202.99%21%21%21%40211b80f717550322996453403e26a5%2112000028806929716%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra</t>
   </si>
 </sst>
 </file>
@@ -602,7 +644,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E5EEACA-D918-4AB7-BE98-0C8D09A79DB9}">
-  <dimension ref="F5:P35"/>
+  <dimension ref="F5:P39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="8" max="9" width="22.88671875" bestFit="1" customWidth="1"/>
@@ -612,30 +654,30 @@
   <sheetData>
     <row r="5" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" t="s">
         <v>18</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>19</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>20</v>
-      </c>
-      <c r="K5" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="6" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F6" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H6" t="s">
         <v>0</v>
@@ -649,10 +691,10 @@
     </row>
     <row r="7" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F7" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H7" t="s">
         <v>2</v>
@@ -666,10 +708,10 @@
     </row>
     <row r="8" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F8" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H8" t="s">
         <v>4</v>
@@ -683,13 +725,13 @@
     </row>
     <row r="9" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F9" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I9">
         <v>5</v>
@@ -703,27 +745,27 @@
     </row>
     <row r="10" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" t="s">
         <v>32</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H10" t="s">
-        <v>35</v>
-      </c>
       <c r="K10" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F11" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I11">
         <v>5</v>
@@ -732,292 +774,296 @@
         <v>5.24</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F12" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H12" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="J12" s="1">
         <v>0.86</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F13" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="J13" s="1">
         <v>2.1800000000000002</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="6:16" x14ac:dyDescent="0.3">
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>29</v>
+      </c>
       <c r="H14" t="s">
-        <v>24</v>
-      </c>
-      <c r="I14">
-        <v>4</v>
-      </c>
-      <c r="J14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K14" t="s">
-        <v>7</v>
+      <c r="J14">
+        <v>1.18</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F15" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H15" t="s">
-        <v>28</v>
-      </c>
-      <c r="J15">
-        <v>1.18</v>
+        <v>7</v>
+      </c>
+      <c r="J15" s="1">
+        <v>2.96</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="P15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="6:16" x14ac:dyDescent="0.3">
       <c r="F16" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H16" t="s">
         <v>8</v>
       </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
       <c r="J16" s="1">
-        <v>2.96</v>
+        <v>2.12</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="6:11" x14ac:dyDescent="0.3">
-      <c r="F17" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>32</v>
-      </c>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
       <c r="H17" t="s">
         <v>9</v>
       </c>
-      <c r="I17">
-        <v>2</v>
-      </c>
-      <c r="J17" s="1">
-        <v>2.12</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>42</v>
-      </c>
+      <c r="J17" s="1"/>
     </row>
     <row r="18" spans="6:11" x14ac:dyDescent="0.3">
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
+      <c r="F18" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>29</v>
+      </c>
       <c r="H18" t="s">
-        <v>10</v>
-      </c>
-      <c r="J18" s="1"/>
+        <v>49</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="19" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F19" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H19" t="s">
+        <v>51</v>
+      </c>
+      <c r="K19" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="20" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F20" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H20" t="s">
-        <v>54</v>
+        <v>11</v>
+      </c>
+      <c r="I20">
+        <v>5</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0.87</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F21" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H21" t="s">
         <v>12</v>
       </c>
       <c r="I21">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J21" s="1">
-        <v>0.87</v>
+        <v>2.38</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F22" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H22" t="s">
         <v>13</v>
       </c>
       <c r="I22">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J22" s="1">
-        <v>2.38</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>44</v>
+        <v>13.63</v>
       </c>
     </row>
     <row r="23" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F23" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H23" t="s">
         <v>14</v>
       </c>
       <c r="I23">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J23" s="1">
-        <v>13.63</v>
+        <v>2.02</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F24" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H24" t="s">
         <v>15</v>
       </c>
-      <c r="I24">
-        <v>10</v>
-      </c>
       <c r="J24" s="1">
-        <v>2.02</v>
+        <v>0.95</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F25" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H25" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="J25" s="1">
-        <v>0.95</v>
+        <v>2.16</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F26" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H26" t="s">
-        <v>29</v>
-      </c>
-      <c r="J26" s="1">
-        <v>2.16</v>
+        <v>16</v>
+      </c>
+      <c r="I26">
+        <v>10</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F27" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H27" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="I27">
         <v>10</v>
       </c>
-      <c r="J27" s="1" t="s">
-        <v>26</v>
+      <c r="J27" s="1">
+        <v>0.87</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F28" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H28" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="I28">
         <v>10</v>
@@ -1026,74 +1072,201 @@
         <v>0.87</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="6:11" x14ac:dyDescent="0.3">
       <c r="F29" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H29" t="s">
-        <v>27</v>
-      </c>
-      <c r="I29">
-        <v>10</v>
+        <v>55</v>
+      </c>
+      <c r="I29" t="s">
+        <v>54</v>
       </c>
       <c r="J29" s="1">
-        <v>0.87</v>
+        <v>12.2</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="6:11" x14ac:dyDescent="0.3">
-      <c r="K30" t="s">
+      <c r="F30" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H30" t="s">
+        <v>57</v>
+      </c>
+      <c r="I30">
+        <v>4</v>
+      </c>
+      <c r="J30" s="1">
+        <v>23.05</v>
+      </c>
+      <c r="K30" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="31" spans="6:11" x14ac:dyDescent="0.3">
+      <c r="F31" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H31" t="s">
+        <v>59</v>
+      </c>
+      <c r="I31">
+        <v>20</v>
+      </c>
+      <c r="J31" s="1">
+        <v>2.0699999999999998</v>
+      </c>
       <c r="K31" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="6:11" x14ac:dyDescent="0.3">
-      <c r="K32" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="35" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="F32" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H32" t="s">
+        <v>61</v>
+      </c>
+      <c r="I32">
+        <v>50</v>
+      </c>
+      <c r="J32" s="1">
+        <v>1.36</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="6:11" x14ac:dyDescent="0.3">
+      <c r="F33" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H33" t="s">
+        <v>63</v>
+      </c>
+      <c r="I33">
+        <v>20</v>
+      </c>
+      <c r="J33" s="1">
+        <v>2.72</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="6:11" x14ac:dyDescent="0.3">
+      <c r="F34" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H34" t="s">
+        <v>65</v>
+      </c>
+      <c r="I34">
+        <v>20</v>
+      </c>
+      <c r="J34" s="1">
+        <v>1.86</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" spans="6:11" x14ac:dyDescent="0.3">
+      <c r="F35" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H35" t="s">
+        <v>69</v>
+      </c>
+      <c r="I35">
+        <v>40</v>
+      </c>
       <c r="J35" s="1">
-        <f>SUM(J6:J29)</f>
-        <v>130.39000000000001</v>
+        <v>4.09</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="36" spans="6:11" x14ac:dyDescent="0.3">
+      <c r="F36" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H36" t="s">
+        <v>70</v>
+      </c>
+      <c r="I36" t="s">
+        <v>68</v>
+      </c>
+      <c r="J36" s="1">
+        <v>3.02</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" spans="6:11" x14ac:dyDescent="0.3">
+      <c r="F37" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H37" t="s">
+        <v>71</v>
+      </c>
+      <c r="I37" t="s">
+        <v>68</v>
+      </c>
+      <c r="J37" s="1">
+        <v>2.99</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="39" spans="6:11" x14ac:dyDescent="0.3">
+      <c r="J39" s="1">
+        <f>SUM(J6:J37)</f>
+        <v>183.75000000000006</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="K16" r:id="rId1" display="https://pt.aliexpress.com/item/1005007492471456.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%209.26%21EUR%202.96%21%21EUR%202.96%21%21%21%402103919917516586444672403e92e2%2112000041009210012%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{D30BACE1-3766-495B-9768-3BCFDBF5A76A}"/>
+    <hyperlink ref="K15" r:id="rId1" display="https://pt.aliexpress.com/item/1005007492471456.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%209.26%21EUR%202.96%21%21EUR%202.96%21%21%21%402103919917516586444672403e92e2%2112000041009210012%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{D30BACE1-3766-495B-9768-3BCFDBF5A76A}"/>
     <hyperlink ref="K9" r:id="rId2" display="https://pt.aliexpress.com/item/1005007671225942.html?spm=a2g0o.productlist.main.4.33bewbpBwbpB4d&amp;algo_pvid=8a0946c9-6135-4953-9734-6fb441ff5631&amp;algo_exp_id=8a0946c9-6135-4953-9734-6fb441ff5631-3&amp;pdp_ext_f=%7B%22order%22%3A%221743%22%2C%22eval%22%3A%221%22%7D&amp;pdp_npi=4%40dis%21EUR%214.83%214.38%21%21%2138.67%2135.07%21%402103867617488812947106565ec0ba%2112000042934077713%21sea%21PT%210%21ABX&amp;curPageLogUid=H76qrjBNJxjg&amp;utparam-url=scene%3Asearch%7Cquery_from%3A" xr:uid="{8ADAAEB6-4FB2-4645-A47C-C2062DBA5048}"/>
     <hyperlink ref="K7" r:id="rId3" xr:uid="{EB473891-DA98-41E5-B720-A8B7A3966362}"/>
     <hyperlink ref="K10" r:id="rId4" display="https://pt.aliexpress.com/item/1005007104356161.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%2014.70%21EUR%207.20%21%21EUR%207.20%21%21%21%402103919917516586444672403e92e2%2112000039414951641%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{A1ED3D8B-594B-4E61-8AC9-026E9C2161CE}"/>
     <hyperlink ref="K11" r:id="rId5" display="https://pt.aliexpress.com/item/1005007539771994.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%2010.73%21EUR%205.15%21%21EUR%205.15%21%21%21%402103919917516586444672403e92e2%2112000048865751738%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{171D51A8-1623-4C5C-8A3F-183D1F3C7276}"/>
     <hyperlink ref="K12" r:id="rId6" display="https://pt.aliexpress.com/item/1005003641187997.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%203.79%21EUR%200.86%21%21EUR%200.86%21%21%21%402103919917516586236261783e92e2%2112000026613929399%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{C7B4A08A-60BA-4F10-BA5C-5B202824838E}"/>
     <hyperlink ref="K13" r:id="rId7" display="https://pt.aliexpress.com/item/1005007285109386.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%2012.41%21EUR%203.73%21%21EUR%203.73%21%21%21%402103919917516586236261783e92e2%2112000040073744618%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{D3DDA1A8-5B23-4F65-B229-C23CCA717BF9}"/>
-    <hyperlink ref="K15" r:id="rId8" display="https://pt.aliexpress.com/item/1005007076787469.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%2010.27%21EUR%202.98%21%21EUR%202.98%21%21%21%402103919917516586444672403e92e2%2112000040125274425%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{BAC729BB-243C-4CA5-AC37-0AD71BB54C02}"/>
-    <hyperlink ref="K17" r:id="rId9" display="https://pt.aliexpress.com/item/1005007038721944.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%203.40%21EUR%203.25%21%21EUR%203.25%21%21%21%402103919917516586236261783e92e2%2112000039181768100%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{ACE1B692-C05F-4C75-8634-F258BBA4FA1A}"/>
-    <hyperlink ref="K21" r:id="rId10" display="https://pt.aliexpress.com/item/1005006293736889.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.61%21EUR%201.64%21%21EUR%201.64%21%21%21%402103919917516586236261783e92e2%2112000036640936680%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{141C7320-160C-43B6-9AD1-561E266872BD}"/>
-    <hyperlink ref="K22" r:id="rId11" display="https://pt.aliexpress.com/item/1005006911573881.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%206.81%21EUR%203.00%21%21EUR%203.00%21%21%21%402103919917516586444672403e92e2%2112000038702556056%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{3B83D5A2-E787-4BB8-8B34-3239F10D54EE}"/>
-    <hyperlink ref="K24" r:id="rId12" display="https://pt.aliexpress.com/item/1005006610500821.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%205.05%21EUR%202.02%21%21EUR%202.02%21%21%21%402103919917516586236261783e92e2%2112000037817952729%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{3460AB49-CD40-4896-8D5B-5CD7AFC73936}"/>
-    <hyperlink ref="K25" r:id="rId13" display="https://pt.aliexpress.com/item/1005008666530101.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%205.72%21EUR%202.63%21%21EUR%202.63%21%21%21%402103919917516586444672403e92e2%2112000046154057678%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{5A529224-1DF5-4D01-A8ED-1E6011C87E7D}"/>
-    <hyperlink ref="K26" r:id="rId14" display="https://pt.aliexpress.com/item/1005003938856402.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.27%21EUR%202.16%21%21EUR%202.16%21%21%21%402103919917516586236261783e92e2%2112000027515454276%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{18A871D0-3BBA-481F-AF6C-D946762EFF1C}"/>
-    <hyperlink ref="K27" r:id="rId15" display="https://pt.aliexpress.com/item/1005001552094086.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%201.22%21EUR%201.22%21%21EUR%201.22%21%21%21%402103919917516586236261783e92e2%2112000016564939105%21ct%21PT%216241319494%21%211%210&amp;pdp_ext_f=%7B%22cart2PdpParams%22%3A%7B%22pdpBusinessMode%22%3A%22retail%22%7D%7D&amp;gatewayAdapt=glo2bra" xr:uid="{11D63B8C-573A-4526-BE92-0589EBB40B60}"/>
-    <hyperlink ref="K28" r:id="rId16" display="https://pt.aliexpress.com/item/1005005699246438.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.00%21EUR%201.91%21%21EUR%201.91%21%21%21%402103919917516586236261783e92e2%2112000034047586751%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{41C7269A-996A-4D4F-90DD-05E4A477CACC}"/>
-    <hyperlink ref="K29" r:id="rId17" display="https://pt.aliexpress.com/item/1005005699246438.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%201.99%21EUR%201.90%21%21EUR%201.90%21%21%21%402103919917516586444672403e92e2%2112000034047586748%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{93A4D611-CE63-49D5-A7E4-F2AD0EED475A}"/>
-    <hyperlink ref="K19" r:id="rId18" display="https://pt.aliexpress.com/item/1005005870392716.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%203.22%21EUR%202.98%21%21EUR%202.98%21%21%21%402103919917516586444672403e92e2%2112000034645748479%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{553B6C49-2B52-4EAC-9A59-F33A5C994A30}"/>
-    <hyperlink ref="K20" r:id="rId19" display="https://pt.aliexpress.com/item/1005006361814667.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%204.13%21EUR%203.88%21%21EUR%203.88%21%21%21%402103919917516586444672403e92e2%2112000036895232315%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{DA9F7222-F361-4477-96B8-073384C3B451}"/>
-    <hyperlink ref="K31" r:id="rId20" display="https://pt.aliexpress.com/item/4000208456751.html?spm=a2g0o.detail.0.0.5d783Gua3Guaba&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.08%21EUR%200.88%21%21EUR%200.88%21%21%21%402103894417539156120946203e3b3f%2110000000799552169%21ct%21PT%21-1%21%211%210&amp;pdp_ext_f=%7B%22cart2PdpParams%22%3A%7B%22pdpBusinessMode%22%3A%22retail%22%7D%7D&amp;gatewayAdapt=glo2bra" xr:uid="{3D2FDB5C-334F-4814-806F-0B9F3FACA477}"/>
+    <hyperlink ref="K14" r:id="rId8" display="https://pt.aliexpress.com/item/1005007076787469.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%2010.27%21EUR%202.98%21%21EUR%202.98%21%21%21%402103919917516586444672403e92e2%2112000040125274425%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{BAC729BB-243C-4CA5-AC37-0AD71BB54C02}"/>
+    <hyperlink ref="K16" r:id="rId9" display="https://pt.aliexpress.com/item/1005007038721944.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%203.40%21EUR%203.25%21%21EUR%203.25%21%21%21%402103919917516586236261783e92e2%2112000039181768100%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{ACE1B692-C05F-4C75-8634-F258BBA4FA1A}"/>
+    <hyperlink ref="K20" r:id="rId10" display="https://pt.aliexpress.com/item/1005006293736889.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.61%21EUR%201.64%21%21EUR%201.64%21%21%21%402103919917516586236261783e92e2%2112000036640936680%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{141C7320-160C-43B6-9AD1-561E266872BD}"/>
+    <hyperlink ref="K21" r:id="rId11" display="https://pt.aliexpress.com/item/1005006911573881.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%206.81%21EUR%203.00%21%21EUR%203.00%21%21%21%402103919917516586444672403e92e2%2112000038702556056%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{3B83D5A2-E787-4BB8-8B34-3239F10D54EE}"/>
+    <hyperlink ref="K23" r:id="rId12" display="https://pt.aliexpress.com/item/1005006610500821.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%205.05%21EUR%202.02%21%21EUR%202.02%21%21%21%402103919917516586236261783e92e2%2112000037817952729%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{3460AB49-CD40-4896-8D5B-5CD7AFC73936}"/>
+    <hyperlink ref="K24" r:id="rId13" display="https://pt.aliexpress.com/item/1005008666530101.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%205.72%21EUR%202.63%21%21EUR%202.63%21%21%21%402103919917516586444672403e92e2%2112000046154057678%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{5A529224-1DF5-4D01-A8ED-1E6011C87E7D}"/>
+    <hyperlink ref="K25" r:id="rId14" display="https://pt.aliexpress.com/item/1005003938856402.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.27%21EUR%202.16%21%21EUR%202.16%21%21%21%402103919917516586236261783e92e2%2112000027515454276%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{18A871D0-3BBA-481F-AF6C-D946762EFF1C}"/>
+    <hyperlink ref="K26" r:id="rId15" display="https://pt.aliexpress.com/item/1005001552094086.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%201.22%21EUR%201.22%21%21EUR%201.22%21%21%21%402103919917516586236261783e92e2%2112000016564939105%21ct%21PT%216241319494%21%211%210&amp;pdp_ext_f=%7B%22cart2PdpParams%22%3A%7B%22pdpBusinessMode%22%3A%22retail%22%7D%7D&amp;gatewayAdapt=glo2bra" xr:uid="{11D63B8C-573A-4526-BE92-0589EBB40B60}"/>
+    <hyperlink ref="K27" r:id="rId16" display="https://pt.aliexpress.com/item/1005005699246438.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.00%21EUR%201.91%21%21EUR%201.91%21%21%21%402103919917516586236261783e92e2%2112000034047586751%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{41C7269A-996A-4D4F-90DD-05E4A477CACC}"/>
+    <hyperlink ref="K28" r:id="rId17" display="https://pt.aliexpress.com/item/1005005699246438.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%201.99%21EUR%201.90%21%21EUR%201.90%21%21%21%402103919917516586444672403e92e2%2112000034047586748%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{93A4D611-CE63-49D5-A7E4-F2AD0EED475A}"/>
+    <hyperlink ref="K18" r:id="rId18" display="https://pt.aliexpress.com/item/1005005870392716.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%203.22%21EUR%202.98%21%21EUR%202.98%21%21%21%402103919917516586444672403e92e2%2112000034645748479%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{553B6C49-2B52-4EAC-9A59-F33A5C994A30}"/>
+    <hyperlink ref="K19" r:id="rId19" display="https://pt.aliexpress.com/item/1005006361814667.html?spm=a2g0o.cart.0.0.2a987f065V31IW&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%204.13%21EUR%203.88%21%21EUR%203.88%21%21%21%402103919917516586444672403e92e2%2112000036895232315%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{DA9F7222-F361-4477-96B8-073384C3B451}"/>
+    <hyperlink ref="K29" r:id="rId20" display="https://pt.aliexpress.com/item/2036819167.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%2018.48%21EUR%2012.20%21%21EUR%2012.20%21%21%21%40211b61a417550327284106006edd2d%2167389781053%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{8D1AB734-C50C-4302-942C-75BE0549B75E}"/>
+    <hyperlink ref="K30" r:id="rId21" display="https://pt.aliexpress.com/item/1005007205148171.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%205.07%21EUR%204.56%21%21EUR%204.56%21%21%21%40211b80f717550322996453403e26a5%2112000039796887787%21ct%21PT%216241319494%21%214%210&amp;gatewayAdapt=glo2bra" xr:uid="{30AE9295-B4FB-4092-8786-3AA3D2504EDD}"/>
+    <hyperlink ref="K31" r:id="rId22" display="https://pt.aliexpress.com/item/1005006897944758.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.07%21EUR%202.07%21%21EUR%202.07%21%21%21%40211b80f717550322996453403e26a5%2112000038652696056%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{08F846F0-B37B-4C73-B068-B744E6144C95}"/>
+    <hyperlink ref="K32" r:id="rId23" display="https://pt.aliexpress.com/item/1005006142488372.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%204.26%21EUR%201.36%21%21EUR%201.36%21%21%21%40211b80f717550322996453403e26a5%2112000035951341855%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{3B09C808-6F25-445E-969F-EDAEC2286184}"/>
+    <hyperlink ref="K33" r:id="rId24" display="https://pt.aliexpress.com/item/32866531235.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%203.05%21EUR%202.72%21%21EUR%202.72%21%21%21%40211b80f717550322996453403e26a5%2112000028848788987%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{DF24833B-98F0-4831-9D0B-42270C693F56}"/>
+    <hyperlink ref="K34" r:id="rId25" display="https://pt.aliexpress.com/item/1005002524973878.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%201.85%21EUR%201.85%21%21EUR%201.85%21%21%21%40211b80f717550322996453403e26a5%2112000020995893453%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{67F09957-E954-4FDA-AF62-E35F22C095D5}"/>
+    <hyperlink ref="K35" r:id="rId26" display="https://pt.aliexpress.com/item/1005003252824475.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%204.37%21EUR%204.09%21%21EUR%204.09%21%21%21%40211b80f717550322996453403e26a5%2112000024867532534%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{77BD1532-CBEA-4F71-9215-0DDF51B19D2A}"/>
+    <hyperlink ref="K36" r:id="rId27" display="https://pt.aliexpress.com/item/1005004336218242.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%203.02%21EUR%203.02%21%21EUR%203.02%21%21%21%40211b80f717550322996453403e26a5%2112000028806929674%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{EFF4DC99-4B5B-4800-B40B-A54E6C800099}"/>
+    <hyperlink ref="K37" r:id="rId28" display="https://pt.aliexpress.com/item/1005004336218242.html?spm=a2g0o.cart.0.0.188c7f06bKYqjx&amp;mp=1&amp;pdp_npi=5%40dis%21EUR%21EUR%202.99%21EUR%202.99%21%21EUR%202.99%21%21%21%40211b80f717550322996453403e26a5%2112000028806929716%21ct%21PT%216241319494%21%211%210&amp;gatewayAdapt=glo2bra" xr:uid="{E7573F72-DEBF-4FC5-948B-CD6929C5561C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId29"/>
 </worksheet>
 </file>
 

</xml_diff>